<commit_message>
site build 2026-10-08 21:32
</commit_message>
<xml_diff>
--- a/models/sovereigns/Senegal_Sovereign_Model.xlsx
+++ b/models/sovereigns/Senegal_Sovereign_Model.xlsx
@@ -647,12 +647,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>09-Sep-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BCEAO Monetary Policy Committee communiqué</t>
+          <t>BCEAO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ANSD, Bulletin Mensuel des Prix à la Consommation Août 2026</t>
+          <t>ANSD</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Aug-26</t>
+          <t>31-Aug-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -736,7 +736,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -784,12 +784,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sep-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Public sector debt, as reconciled by Cour des Comptes audit with IMF technical assistance (previously reported ~74%)</t>
+          <t>Public debt, ~132% of GDP at end-2024 against ~74% previously reported; attribution (Cour des Comptes Feb-25 vs later IMF reconciliation) unresolved</t>
         </is>
       </c>
     </row>
@@ -839,11 +839,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -925,11 +921,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1097,11 +1089,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1266,7 +1254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Successor financing arrangement (staff-level agreement) replacing suspended EFF/ECF approved Jun-23</t>
+          <t>Staff-level agreement on new arrangement replacing suspended $1.8B facility</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1274,7 +1262,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>15-Dec-26 (Executive Board consideration)</t>
+          <t>Executive Board consideration 15-Dec-26</t>
         </is>
       </c>
     </row>
@@ -1336,8 +1324,14 @@
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="E2" s="2" t="n">
+        <v>40.469</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1355,7 +1349,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ANSD / IMF, Sep-26</t>
+          <t>ANSD / IMF, 08-Oct-26</t>
         </is>
       </c>
     </row>
@@ -1380,8 +1374,14 @@
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="E5" s="2" t="n">
+        <v>-6.2</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1392,8 +1392,14 @@
       <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="E6" s="2" t="n">
+        <v>-6.7</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1423,7 +1429,7 @@
       <c r="E8" s="2" t="n"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Cour des Comptes / IMF, Sep-26 (public sector debt, reconciled)</t>
+          <t>Cour des Comptes / IMF, 08-Oct-26</t>
         </is>
       </c>
     </row>

</xml_diff>